<commit_message>
Updated CHE_grids model - 2025-09-07 00:03
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8BD231E-53F1-477B-9F30-D6547477FE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8A2F99C-11ED-40FE-90BE-EF0C9D111364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5270,7 +5270,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA00301-2FF6-4533-878B-82DA0FECC4F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA0B652E-CCE1-45C0-82C2-80892F551D54}">
   <dimension ref="B9:D191"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7287,7 +7287,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{730EB7E4-D14B-43F6-A32B-293B2C5EC513}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16DB4A1A-EDD3-4FAD-90D4-7CDB48079C79}">
   <dimension ref="B2:D184"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE_grids model - 2025-09-07 23:31
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8A2F99C-11ED-40FE-90BE-EF0C9D111364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC6D6437-FC37-43C8-9DDA-808F10CA80A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5270,7 +5270,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA0B652E-CCE1-45C0-82C2-80892F551D54}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57309AC4-3703-4DE2-BB23-03B5C36CFC29}">
   <dimension ref="B9:D191"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7011,10 +7011,10 @@
         <v>454</v>
       </c>
       <c r="C167">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D167">
-        <v>6.2896976410000001</v>
+        <v>6.289697641356212</v>
       </c>
     </row>
     <row r="168" spans="2:4">
@@ -7022,10 +7022,10 @@
         <v>455</v>
       </c>
       <c r="C168">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D168">
-        <v>6.2896976410000001</v>
+        <v>6.289697641356212</v>
       </c>
     </row>
     <row r="169" spans="2:4">
@@ -7033,10 +7033,10 @@
         <v>456</v>
       </c>
       <c r="C169">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D169">
-        <v>6.2896976410000001</v>
+        <v>6.289697641356212</v>
       </c>
     </row>
     <row r="170" spans="2:4">
@@ -7044,10 +7044,10 @@
         <v>457</v>
       </c>
       <c r="C170">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D170">
-        <v>6.9349650939999998</v>
+        <v>6.9349650942374748</v>
       </c>
     </row>
     <row r="171" spans="2:4">
@@ -7055,10 +7055,10 @@
         <v>458</v>
       </c>
       <c r="C171">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D171">
-        <v>6.9349650939999998</v>
+        <v>6.9349650942374748</v>
       </c>
     </row>
     <row r="172" spans="2:4">
@@ -7066,10 +7066,10 @@
         <v>459</v>
       </c>
       <c r="C172">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D172">
-        <v>6.9349650939999998</v>
+        <v>6.9349650942374748</v>
       </c>
     </row>
     <row r="173" spans="2:4">
@@ -7077,10 +7077,10 @@
         <v>460</v>
       </c>
       <c r="C173">
-        <v>47.48699027</v>
+        <v>47.486990272793413</v>
       </c>
       <c r="D173">
-        <v>6.9349650939999998</v>
+        <v>6.9349650942374748</v>
       </c>
     </row>
     <row r="174" spans="2:4">
@@ -7088,10 +7088,10 @@
         <v>461</v>
       </c>
       <c r="C174">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D174">
-        <v>7.5802325469999996</v>
+        <v>7.5802325471187393</v>
       </c>
     </row>
     <row r="175" spans="2:4">
@@ -7099,10 +7099,10 @@
         <v>462</v>
       </c>
       <c r="C175">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D175">
-        <v>7.5802325469999996</v>
+        <v>7.5802325471187393</v>
       </c>
     </row>
     <row r="176" spans="2:4">
@@ -7110,10 +7110,10 @@
         <v>463</v>
       </c>
       <c r="C176">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D176">
-        <v>7.5802325469999996</v>
+        <v>7.5802325471187393</v>
       </c>
     </row>
     <row r="177" spans="2:4">
@@ -7121,10 +7121,10 @@
         <v>464</v>
       </c>
       <c r="C177">
-        <v>47.48699027</v>
+        <v>47.486990272793413</v>
       </c>
       <c r="D177">
-        <v>7.5802325469999996</v>
+        <v>7.5802325471187393</v>
       </c>
     </row>
     <row r="178" spans="2:4">
@@ -7132,10 +7132,10 @@
         <v>465</v>
       </c>
       <c r="C178">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D178">
-        <v>8.2255000000000003</v>
+        <v>8.225500000000002</v>
       </c>
     </row>
     <row r="179" spans="2:4">
@@ -7143,10 +7143,10 @@
         <v>466</v>
       </c>
       <c r="C179">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D179">
-        <v>8.2255000000000003</v>
+        <v>8.225500000000002</v>
       </c>
     </row>
     <row r="180" spans="2:4">
@@ -7154,10 +7154,10 @@
         <v>467</v>
       </c>
       <c r="C180">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D180">
-        <v>8.2255000000000003</v>
+        <v>8.225500000000002</v>
       </c>
     </row>
     <row r="181" spans="2:4">
@@ -7165,10 +7165,10 @@
         <v>468</v>
       </c>
       <c r="C181">
-        <v>47.48699027</v>
+        <v>47.486990272793413</v>
       </c>
       <c r="D181">
-        <v>8.2255000000000003</v>
+        <v>8.225500000000002</v>
       </c>
     </row>
     <row r="182" spans="2:4">
@@ -7176,10 +7176,10 @@
         <v>469</v>
       </c>
       <c r="C182">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D182">
-        <v>8.8707674529999991</v>
+        <v>8.8707674528812674</v>
       </c>
     </row>
     <row r="183" spans="2:4">
@@ -7187,10 +7187,10 @@
         <v>470</v>
       </c>
       <c r="C183">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D183">
-        <v>8.8707674529999991</v>
+        <v>8.8707674528812674</v>
       </c>
     </row>
     <row r="184" spans="2:4">
@@ -7198,10 +7198,10 @@
         <v>471</v>
       </c>
       <c r="C184">
-        <v>47.48699027</v>
+        <v>47.486990272793413</v>
       </c>
       <c r="D184">
-        <v>8.8707674529999991</v>
+        <v>8.8707674528812674</v>
       </c>
     </row>
     <row r="185" spans="2:4">
@@ -7209,10 +7209,10 @@
         <v>472</v>
       </c>
       <c r="C185">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D185">
-        <v>9.5160349059999998</v>
+        <v>9.5160349057625293</v>
       </c>
     </row>
     <row r="186" spans="2:4">
@@ -7220,10 +7220,10 @@
         <v>473</v>
       </c>
       <c r="C186">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D186">
-        <v>9.5160349059999998</v>
+        <v>9.5160349057625293</v>
       </c>
     </row>
     <row r="187" spans="2:4">
@@ -7231,10 +7231,10 @@
         <v>474</v>
       </c>
       <c r="C187">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D187">
-        <v>9.5160349059999998</v>
+        <v>9.5160349057625293</v>
       </c>
     </row>
     <row r="188" spans="2:4">
@@ -7242,10 +7242,10 @@
         <v>475</v>
       </c>
       <c r="C188">
-        <v>47.48699027</v>
+        <v>47.486990272793413</v>
       </c>
       <c r="D188">
-        <v>9.5160349059999998</v>
+        <v>9.5160349057625293</v>
       </c>
     </row>
     <row r="189" spans="2:4">
@@ -7253,10 +7253,10 @@
         <v>476</v>
       </c>
       <c r="C189">
-        <v>46.13800973</v>
+        <v>46.138009727206594</v>
       </c>
       <c r="D189">
-        <v>10.161302360000001</v>
+        <v>10.161302358643791</v>
       </c>
     </row>
     <row r="190" spans="2:4">
@@ -7264,10 +7264,10 @@
         <v>477</v>
       </c>
       <c r="C190">
-        <v>46.587669910000002</v>
+        <v>46.587669909068872</v>
       </c>
       <c r="D190">
-        <v>10.161302360000001</v>
+        <v>10.161302358643791</v>
       </c>
     </row>
     <row r="191" spans="2:4">
@@ -7275,10 +7275,10 @@
         <v>478</v>
       </c>
       <c r="C191">
-        <v>47.037330089999998</v>
+        <v>47.037330090931135</v>
       </c>
       <c r="D191">
-        <v>10.161302360000001</v>
+        <v>10.161302358643791</v>
       </c>
     </row>
   </sheetData>
@@ -7287,7 +7287,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16DB4A1A-EDD3-4FAD-90D4-7CDB48079C79}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC06C61E-6B66-4FC8-9526-1932D145970C}">
   <dimension ref="B2:D184"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE_grids model - 2025-09-08 23:26
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3FE111B-61E9-4B35-BEBB-358F699A353D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{756201FA-8E40-4495-A8B5-18149CF1D974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7620,7 +7620,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297FE9BD-F357-45F8-8B76-EC0D919201F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ACE3B64-9282-4696-9453-AE6DBD840B21}">
   <dimension ref="B9:D191"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9637,7 +9637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{532C3B3F-D7CF-4098-BECC-6CFBFBF7AF92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B7D065F-590E-46B7-A4C4-B93B764C60E5}">
   <dimension ref="B2:D184"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE_grids model - 2025-09-09 00:22
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHE_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{756201FA-8E40-4495-A8B5-18149CF1D974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1385FB93-2A09-4918-9009-91A36D020CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7620,7 +7620,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ACE3B64-9282-4696-9453-AE6DBD840B21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2956C458-788B-413F-BC1B-A343B65292BD}">
   <dimension ref="B9:D191"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9637,7 +9637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B7D065F-590E-46B7-A4C4-B93B764C60E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE8CEA5-F12D-4C98-88D1-876BAA6D0A49}">
   <dimension ref="B2:D184"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>